<commit_message>
Bug fixes, trainers and AI work
</commit_message>
<xml_diff>
--- a/stuff/xhenos story work.xlsx
+++ b/stuff/xhenos story work.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\git\PokemonXhenos\stuff\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76BD549C-2F1B-4B4B-AE93-E2D6B14EA595}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE757816-1563-4C6C-8A69-2C1702CD2B84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{271A13BE-4517-4656-AED4-3C6BEDDB1427}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="437" uniqueCount="399">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="400">
   <si>
     <t>Current</t>
   </si>
@@ -1233,6 +1233,9 @@
   </si>
   <si>
     <t>Deletor</t>
+  </si>
+  <si>
+    <t>Move Enc</t>
   </si>
 </sst>
 </file>
@@ -2257,6 +2260,9 @@
       <c r="L29" t="s">
         <v>392</v>
       </c>
+      <c r="M29" t="s">
+        <v>399</v>
+      </c>
     </row>
     <row r="30" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" t="s">

</xml_diff>

<commit_message>
Work on settings, new sprite and got Extreme Mode lead selection done!
</commit_message>
<xml_diff>
--- a/stuff/xhenos story work.xlsx
+++ b/stuff/xhenos story work.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\git\PokemonXhenos\stuff\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C96073F-56AC-480D-BB42-1BAC4548B5F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0505CEFF-85EA-4B52-9A87-4835CC3C797B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{271A13BE-4517-4656-AED4-3C6BEDDB1427}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{271A13BE-4517-4656-AED4-3C6BEDDB1427}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="400">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="401">
   <si>
     <t>Current</t>
   </si>
@@ -1236,6 +1236,9 @@
   </si>
   <si>
     <t>Move Enc</t>
+  </si>
+  <si>
+    <t>Set Difficulty</t>
   </si>
 </sst>
 </file>
@@ -2009,6 +2012,9 @@
       <c r="AB25" t="s">
         <v>371</v>
       </c>
+      <c r="AC25" t="s">
+        <v>400</v>
+      </c>
     </row>
     <row r="26" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" t="s">

</xml_diff>

<commit_message>
Bug fixes for the new update
</commit_message>
<xml_diff>
--- a/stuff/xhenos story work.xlsx
+++ b/stuff/xhenos story work.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\git\PokemonXhenos\stuff\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0505CEFF-85EA-4B52-9A87-4835CC3C797B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0B5168A-9781-498D-A03C-A86FFF118D31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{271A13BE-4517-4656-AED4-3C6BEDDB1427}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="401">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="880" uniqueCount="402">
   <si>
     <t>Current</t>
   </si>
@@ -1239,6 +1239,9 @@
   </si>
   <si>
     <t>Set Difficulty</t>
+  </si>
+  <si>
+    <t>Rick Pad</t>
   </si>
 </sst>
 </file>
@@ -2316,6 +2319,9 @@
       <c r="O30" t="s">
         <v>322</v>
       </c>
+      <c r="P30" t="s">
+        <v>401</v>
+      </c>
     </row>
     <row r="31" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" t="s">

</xml_diff>

<commit_message>
2 new sprites and tons of changes during Italy 2-week trip!
</commit_message>
<xml_diff>
--- a/stuff/xhenos story work.xlsx
+++ b/stuff/xhenos story work.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\git\PokemonXhenos\stuff\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shaej\git\PokemonGame\stuff\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0B5168A-9781-498D-A03C-A86FFF118D31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CB33463-B411-473B-96B2-803165345FC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{271A13BE-4517-4656-AED4-3C6BEDDB1427}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{271A13BE-4517-4656-AED4-3C6BEDDB1427}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="880" uniqueCount="402">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="445" uniqueCount="407">
   <si>
     <t>Current</t>
   </si>
@@ -1242,6 +1242,21 @@
   </si>
   <si>
     <t>Rick Pad</t>
+  </si>
+  <si>
+    <t>Whiskeroar</t>
+  </si>
+  <si>
+    <t>Chlorie</t>
+  </si>
+  <si>
+    <t>Astrid</t>
+  </si>
+  <si>
+    <t>Arthra</t>
+  </si>
+  <si>
+    <t>Necrozma can be obtained once the player rematches the league and wins again, then after beating Ryder again he will have Necrozma call more of its kind by the ship in space</t>
   </si>
 </sst>
 </file>
@@ -1619,15 +1634,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5853A869-EFC3-49CB-8DC6-87B1B6715E26}">
-  <dimension ref="A1:AD154"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AD155"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="47" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="165" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="9.42578125" customWidth="1"/>
+    <col min="17" max="17" width="9.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1638,7 +1653,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -1649,7 +1664,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -1657,7 +1672,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1665,7 +1680,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -1676,7 +1691,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -1687,7 +1702,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -1695,7 +1710,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -1703,7 +1718,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -1711,7 +1726,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -1719,7 +1734,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>12</v>
       </c>
@@ -1727,7 +1742,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -1735,7 +1750,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>13</v>
       </c>
@@ -1743,7 +1758,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>14</v>
       </c>
@@ -1751,7 +1766,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>15</v>
       </c>
@@ -1759,7 +1774,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>16</v>
       </c>
@@ -1767,7 +1782,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="17" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>17</v>
       </c>
@@ -1778,7 +1793,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="18" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>18</v>
       </c>
@@ -1789,7 +1804,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="19" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>19</v>
       </c>
@@ -1800,7 +1815,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="20" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>20</v>
       </c>
@@ -1811,7 +1826,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="21" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>21</v>
       </c>
@@ -1822,7 +1837,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="22" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>22</v>
       </c>
@@ -1830,7 +1845,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="23" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>23</v>
       </c>
@@ -1838,7 +1853,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="24" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>24</v>
       </c>
@@ -1930,7 +1945,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="25" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>25</v>
       </c>
@@ -2019,7 +2034,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="26" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>26</v>
       </c>
@@ -2111,7 +2126,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="27" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>27</v>
       </c>
@@ -2176,7 +2191,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="28" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>28</v>
       </c>
@@ -2232,7 +2247,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="29" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>29</v>
       </c>
@@ -2273,7 +2288,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="30" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>30</v>
       </c>
@@ -2323,7 +2338,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="31" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>31</v>
       </c>
@@ -2397,7 +2412,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="32" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>32</v>
       </c>
@@ -2489,7 +2504,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="33" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>33</v>
       </c>
@@ -2548,7 +2563,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="34" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>34</v>
       </c>
@@ -2564,8 +2579,20 @@
       <c r="E34" s="2" t="s">
         <v>244</v>
       </c>
-    </row>
-    <row r="35" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="K34" t="s">
+        <v>402</v>
+      </c>
+      <c r="L34" t="s">
+        <v>403</v>
+      </c>
+      <c r="M34" t="s">
+        <v>404</v>
+      </c>
+      <c r="N34" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="35" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>35</v>
       </c>
@@ -2579,7 +2606,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="36" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>36</v>
       </c>
@@ -2593,7 +2620,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="37" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>37</v>
       </c>
@@ -2607,7 +2634,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="38" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>39</v>
       </c>
@@ -2621,7 +2648,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="39" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>38</v>
       </c>
@@ -2635,7 +2662,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="40" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>40</v>
       </c>
@@ -2649,7 +2676,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="41" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>41</v>
       </c>
@@ -2663,7 +2690,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="42" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>42</v>
       </c>
@@ -2677,7 +2704,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="43" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>45</v>
       </c>
@@ -2691,7 +2718,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="44" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>43</v>
       </c>
@@ -2705,7 +2732,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="45" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>44</v>
       </c>
@@ -2719,7 +2746,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="46" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>46</v>
       </c>
@@ -2733,7 +2760,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="47" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>47</v>
       </c>
@@ -2747,7 +2774,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="48" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>51</v>
       </c>
@@ -2761,7 +2788,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>52</v>
       </c>
@@ -2775,7 +2802,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>48</v>
       </c>
@@ -2789,7 +2816,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>49</v>
       </c>
@@ -2803,7 +2830,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>50</v>
       </c>
@@ -2817,7 +2844,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>53</v>
       </c>
@@ -2831,7 +2858,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>54</v>
       </c>
@@ -2845,7 +2872,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>55</v>
       </c>
@@ -2859,7 +2886,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>56</v>
       </c>
@@ -2873,7 +2900,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>57</v>
       </c>
@@ -2887,7 +2914,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>58</v>
       </c>
@@ -2901,7 +2928,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>61</v>
       </c>
@@ -2915,7 +2942,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>59</v>
       </c>
@@ -2929,7 +2956,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>60</v>
       </c>
@@ -2937,7 +2964,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>62</v>
       </c>
@@ -2945,7 +2972,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>63</v>
       </c>
@@ -2953,7 +2980,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>64</v>
       </c>
@@ -2961,7 +2988,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>65</v>
       </c>
@@ -2969,7 +2996,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>66</v>
       </c>
@@ -2977,7 +3004,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>67</v>
       </c>
@@ -2985,7 +3012,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>68</v>
       </c>
@@ -2993,7 +3020,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>69</v>
       </c>
@@ -3001,7 +3028,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>70</v>
       </c>
@@ -3009,7 +3036,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>71</v>
       </c>
@@ -3017,7 +3044,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>72</v>
       </c>
@@ -3025,7 +3052,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>73</v>
       </c>
@@ -3033,7 +3060,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>74</v>
       </c>
@@ -3041,7 +3068,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>75</v>
       </c>
@@ -3049,7 +3076,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>76</v>
       </c>
@@ -3057,7 +3084,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>77</v>
       </c>
@@ -3065,7 +3092,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>78</v>
       </c>
@@ -3073,7 +3100,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>79</v>
       </c>
@@ -3081,7 +3108,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>80</v>
       </c>
@@ -3089,7 +3116,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>81</v>
       </c>
@@ -3097,7 +3124,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>82</v>
       </c>
@@ -3105,17 +3132,17 @@
         <v>143</v>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B83" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B84" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B85" t="s">
         <v>145</v>
       </c>
@@ -3123,349 +3150,354 @@
         <v>154</v>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B86" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B87" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B88" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B89" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B90" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B91" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B92" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B93" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B94" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B95" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B96" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="97" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="97" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B97" t="s">
         <v>323</v>
       </c>
     </row>
-    <row r="98" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="98" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B98" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="99" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="99" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B99" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="100" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="100" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B100" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="101" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="101" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B101" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="102" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="102" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B102" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="103" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="103" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B103" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="104" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="104" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B104" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="105" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="105" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B105" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="106" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="106" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B106" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="107" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="107" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B107" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="108" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="108" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B108" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="109" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="109" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B109" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="110" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="110" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B110" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="111" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="111" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B111" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="112" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="112" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B112" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="113" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="113" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B113" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="114" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="114" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B114" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="115" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="115" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B115" t="s">
         <v>320</v>
       </c>
     </row>
-    <row r="116" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="116" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B116" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="117" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="117" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B117" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="118" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="118" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B118" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="119" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="119" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B119" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="120" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="120" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B120" t="s">
         <v>373</v>
       </c>
     </row>
-    <row r="121" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="121" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B121" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="122" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="122" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B122" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="123" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="123" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B123" t="s">
         <v>374</v>
       </c>
     </row>
-    <row r="124" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="124" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B124" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="125" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="125" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B125" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="126" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="126" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B126" t="s">
         <v>375</v>
       </c>
     </row>
-    <row r="127" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="127" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B127" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="128" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="128" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B128" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="129" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="129" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B129" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="130" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="130" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B130" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="131" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="131" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B131" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="132" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="132" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B132" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="133" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="133" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B133" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="134" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="134" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B134" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="135" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="135" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B135" t="s">
         <v>325</v>
       </c>
     </row>
-    <row r="136" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="136" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B136" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="137" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="137" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B137" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="138" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="138" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B138" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="139" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="139" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B139" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="140" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="140" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B140" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="141" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="141" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B141" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="142" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="142" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B142" t="s">
         <v>196</v>
       </c>
     </row>
-    <row r="143" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="143" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B143" t="s">
         <v>380</v>
       </c>
     </row>
-    <row r="144" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="144" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B144" t="s">
         <v>381</v>
       </c>
     </row>
-    <row r="145" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="145" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B145" t="s">
         <v>382</v>
       </c>
     </row>
-    <row r="146" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="146" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B146" t="s">
         <v>383</v>
       </c>
     </row>
-    <row r="147" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="147" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B147" t="s">
         <v>384</v>
       </c>
     </row>
-    <row r="148" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="148" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B148" t="s">
         <v>385</v>
       </c>
     </row>
-    <row r="149" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="149" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B149" t="s">
         <v>386</v>
       </c>
     </row>
-    <row r="150" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="150" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B150" t="s">
         <v>387</v>
       </c>
     </row>
-    <row r="151" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="151" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B151" t="s">
         <v>388</v>
       </c>
     </row>
-    <row r="152" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="152" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B152" t="s">
         <v>389</v>
       </c>
     </row>
-    <row r="153" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="153" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B153" t="s">
         <v>390</v>
       </c>
     </row>
-    <row r="154" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="154" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B154" t="s">
         <v>391</v>
+      </c>
+    </row>
+    <row r="155" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B155" t="s">
+        <v>406</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
New sprite, Magic move animations and finished Bug move animations!
</commit_message>
<xml_diff>
--- a/stuff/xhenos story work.xlsx
+++ b/stuff/xhenos story work.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shaej\git\PokemonGame\stuff\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\git\PokemonXhenos\stuff\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CB33463-B411-473B-96B2-803165345FC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C6C0D95-6AB4-4F52-BE87-D25DEB2AFE9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{271A13BE-4517-4656-AED4-3C6BEDDB1427}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{271A13BE-4517-4656-AED4-3C6BEDDB1427}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="445" uniqueCount="407">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="446" uniqueCount="408">
   <si>
     <t>Current</t>
   </si>
@@ -1257,6 +1257,9 @@
   </si>
   <si>
     <t>Necrozma can be obtained once the player rematches the league and wins again, then after beating Ryder again he will have Necrozma call more of its kind by the ship in space</t>
+  </si>
+  <si>
+    <t>Third Starter</t>
   </si>
 </sst>
 </file>
@@ -1635,14 +1638,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5853A869-EFC3-49CB-8DC6-87B1B6715E26}">
   <dimension ref="A1:AD155"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="47" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="165" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="9.44140625" customWidth="1"/>
+    <col min="17" max="17" width="9.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1653,7 +1656,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -1664,7 +1667,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -1672,7 +1675,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1680,7 +1683,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -1691,7 +1694,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -1702,7 +1705,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -1710,7 +1713,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -1718,7 +1721,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -1726,7 +1729,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -1734,7 +1737,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>12</v>
       </c>
@@ -1742,7 +1745,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -1750,7 +1753,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>13</v>
       </c>
@@ -1758,7 +1761,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>14</v>
       </c>
@@ -1766,7 +1769,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>15</v>
       </c>
@@ -1774,7 +1777,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>16</v>
       </c>
@@ -1782,7 +1785,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="17" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>17</v>
       </c>
@@ -1793,7 +1796,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="18" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>18</v>
       </c>
@@ -1804,7 +1807,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="19" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>19</v>
       </c>
@@ -1815,7 +1818,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="20" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>20</v>
       </c>
@@ -1826,7 +1829,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="21" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>21</v>
       </c>
@@ -1837,7 +1840,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="22" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>22</v>
       </c>
@@ -1845,7 +1848,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="23" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>23</v>
       </c>
@@ -1853,7 +1856,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="24" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>24</v>
       </c>
@@ -1945,7 +1948,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="25" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>25</v>
       </c>
@@ -2034,7 +2037,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="26" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>26</v>
       </c>
@@ -2126,7 +2129,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="27" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>27</v>
       </c>
@@ -2191,7 +2194,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="28" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>28</v>
       </c>
@@ -2247,7 +2250,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="29" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>29</v>
       </c>
@@ -2288,7 +2291,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="30" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>30</v>
       </c>
@@ -2338,7 +2341,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="31" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>31</v>
       </c>
@@ -2412,7 +2415,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="32" spans="1:30" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>32</v>
       </c>
@@ -2504,7 +2507,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="33" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>33</v>
       </c>
@@ -2562,8 +2565,11 @@
       <c r="S33" t="s">
         <v>396</v>
       </c>
-    </row>
-    <row r="34" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="T33" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="34" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>34</v>
       </c>
@@ -2592,7 +2598,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="35" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>35</v>
       </c>
@@ -2606,7 +2612,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="36" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>36</v>
       </c>
@@ -2620,7 +2626,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="37" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>37</v>
       </c>
@@ -2634,7 +2640,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="38" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>39</v>
       </c>
@@ -2648,7 +2654,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="39" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>38</v>
       </c>
@@ -2662,7 +2668,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="40" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>40</v>
       </c>
@@ -2676,7 +2682,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="41" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>41</v>
       </c>
@@ -2690,7 +2696,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="42" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>42</v>
       </c>
@@ -2704,7 +2710,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="43" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>45</v>
       </c>
@@ -2718,7 +2724,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="44" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>43</v>
       </c>
@@ -2732,7 +2738,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="45" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>44</v>
       </c>
@@ -2746,7 +2752,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="46" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>46</v>
       </c>
@@ -2760,7 +2766,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="47" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>47</v>
       </c>
@@ -2774,7 +2780,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="48" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>51</v>
       </c>
@@ -2788,7 +2794,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>52</v>
       </c>
@@ -2802,7 +2808,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>48</v>
       </c>
@@ -2816,7 +2822,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>49</v>
       </c>
@@ -2830,7 +2836,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>50</v>
       </c>
@@ -2844,7 +2850,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>53</v>
       </c>
@@ -2858,7 +2864,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>54</v>
       </c>
@@ -2872,7 +2878,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>55</v>
       </c>
@@ -2886,7 +2892,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>56</v>
       </c>
@@ -2900,7 +2906,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>57</v>
       </c>
@@ -2914,7 +2920,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>58</v>
       </c>
@@ -2928,7 +2934,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>61</v>
       </c>
@@ -2942,7 +2948,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>59</v>
       </c>
@@ -2956,7 +2962,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>60</v>
       </c>
@@ -2964,7 +2970,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>62</v>
       </c>
@@ -2972,7 +2978,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>63</v>
       </c>
@@ -2980,7 +2986,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>64</v>
       </c>
@@ -2988,7 +2994,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>65</v>
       </c>
@@ -2996,7 +3002,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>66</v>
       </c>
@@ -3004,7 +3010,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>67</v>
       </c>
@@ -3012,7 +3018,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>68</v>
       </c>
@@ -3020,7 +3026,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>69</v>
       </c>
@@ -3028,7 +3034,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>70</v>
       </c>
@@ -3036,7 +3042,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>71</v>
       </c>
@@ -3044,7 +3050,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>72</v>
       </c>
@@ -3052,7 +3058,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>73</v>
       </c>
@@ -3060,7 +3066,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>74</v>
       </c>
@@ -3068,7 +3074,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>75</v>
       </c>
@@ -3076,7 +3082,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>76</v>
       </c>
@@ -3084,7 +3090,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>77</v>
       </c>
@@ -3092,7 +3098,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>78</v>
       </c>
@@ -3100,7 +3106,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>79</v>
       </c>
@@ -3108,7 +3114,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>80</v>
       </c>
@@ -3116,7 +3122,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>81</v>
       </c>
@@ -3124,7 +3130,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>82</v>
       </c>
@@ -3132,17 +3138,17 @@
         <v>143</v>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B83" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B84" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B85" t="s">
         <v>145</v>
       </c>
@@ -3150,352 +3156,352 @@
         <v>154</v>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B86" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B87" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B88" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B89" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B90" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B91" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B92" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B93" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B94" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B95" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B96" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="97" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="97" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B97" t="s">
         <v>323</v>
       </c>
     </row>
-    <row r="98" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="98" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B98" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="99" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="99" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B99" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="100" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="100" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B100" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="101" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="101" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B101" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="102" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="102" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B102" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="103" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="103" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B103" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="104" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="104" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B104" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="105" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="105" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B105" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="106" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="106" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B106" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="107" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="107" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B107" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="108" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="108" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B108" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="109" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="109" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B109" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="110" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="110" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B110" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="111" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="111" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B111" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="112" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="112" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B112" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="113" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="113" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B113" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="114" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="114" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B114" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="115" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="115" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B115" t="s">
         <v>320</v>
       </c>
     </row>
-    <row r="116" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="116" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B116" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="117" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="117" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B117" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="118" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="118" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B118" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="119" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="119" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B119" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="120" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="120" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B120" t="s">
         <v>373</v>
       </c>
     </row>
-    <row r="121" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="121" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B121" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="122" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="122" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B122" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="123" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="123" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B123" t="s">
         <v>374</v>
       </c>
     </row>
-    <row r="124" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="124" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B124" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="125" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="125" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B125" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="126" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="126" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B126" t="s">
         <v>375</v>
       </c>
     </row>
-    <row r="127" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="127" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B127" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="128" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="128" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B128" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="129" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="129" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B129" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="130" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="130" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B130" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="131" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="131" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B131" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="132" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="132" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B132" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="133" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="133" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B133" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="134" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="134" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B134" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="135" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="135" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B135" t="s">
         <v>325</v>
       </c>
     </row>
-    <row r="136" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="136" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B136" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="137" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="137" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B137" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="138" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="138" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B138" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="139" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="139" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B139" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="140" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="140" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B140" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="141" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="141" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B141" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="142" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="142" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B142" t="s">
         <v>196</v>
       </c>
     </row>
-    <row r="143" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="143" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B143" t="s">
         <v>380</v>
       </c>
     </row>
-    <row r="144" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="144" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B144" t="s">
         <v>381</v>
       </c>
     </row>
-    <row r="145" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="145" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B145" t="s">
         <v>382</v>
       </c>
     </row>
-    <row r="146" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="146" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B146" t="s">
         <v>383</v>
       </c>
     </row>
-    <row r="147" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="147" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B147" t="s">
         <v>384</v>
       </c>
     </row>
-    <row r="148" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="148" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B148" t="s">
         <v>385</v>
       </c>
     </row>
-    <row r="149" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="149" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B149" t="s">
         <v>386</v>
       </c>
     </row>
-    <row r="150" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="150" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B150" t="s">
         <v>387</v>
       </c>
     </row>
-    <row r="151" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="151" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B151" t="s">
         <v>388</v>
       </c>
     </row>
-    <row r="152" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="152" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B152" t="s">
         <v>389</v>
       </c>
     </row>
-    <row r="153" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="153" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B153" t="s">
         <v>390</v>
       </c>
     </row>
-    <row r="154" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="154" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B154" t="s">
         <v>391</v>
       </c>
     </row>
-    <row r="155" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="155" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B155" t="s">
         <v>406</v>
       </c>

</xml_diff>

<commit_message>
Bug fixes, new sprite and 4th E4 room done!
</commit_message>
<xml_diff>
--- a/stuff/xhenos story work.xlsx
+++ b/stuff/xhenos story work.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\git\PokemonXhenos\stuff\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C6C0D95-6AB4-4F52-BE87-D25DEB2AFE9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC8EA829-FD4E-4FBA-B8ED-E851A110DBD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{271A13BE-4517-4656-AED4-3C6BEDDB1427}"/>
   </bookViews>
@@ -614,9 +614,6 @@
     <t>Since you won't give up yours she realizes its either have both or none, she feels like she's worthy enough without it and sets it back to its home</t>
   </si>
   <si>
-    <t>Then Nova pulls up to personally thank you guys for setting her free, she gives you both an ability patch, and you all go into the champion room</t>
-  </si>
-  <si>
     <t>You all are surprised to see Ryder in there talking/battling the champion, not only alive but he has Necrozma now</t>
   </si>
   <si>
@@ -1260,6 +1257,9 @@
   </si>
   <si>
     <t>Third Starter</t>
+  </si>
+  <si>
+    <t>Then Nova pulls up to personally thank you guys for setting her free and you all go into the champion room</t>
   </si>
 </sst>
 </file>
@@ -1653,7 +1653,7 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -1790,10 +1790,10 @@
         <v>17</v>
       </c>
       <c r="B17" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="Z17" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="18" spans="1:30" x14ac:dyDescent="0.25">
@@ -1804,7 +1804,7 @@
         <v>91</v>
       </c>
       <c r="Z18" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="19" spans="1:30" x14ac:dyDescent="0.25">
@@ -1815,7 +1815,7 @@
         <v>92</v>
       </c>
       <c r="Z19" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="20" spans="1:30" x14ac:dyDescent="0.25">
@@ -1826,7 +1826,7 @@
         <v>93</v>
       </c>
       <c r="Z20" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="21" spans="1:30" x14ac:dyDescent="0.25">
@@ -1834,10 +1834,10 @@
         <v>21</v>
       </c>
       <c r="B21" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="Z21" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="22" spans="1:30" x14ac:dyDescent="0.25">
@@ -1845,7 +1845,7 @@
         <v>22</v>
       </c>
       <c r="B22" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="23" spans="1:30" x14ac:dyDescent="0.25">
@@ -1867,10 +1867,10 @@
         <v>0</v>
       </c>
       <c r="D24" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E24" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="F24">
         <v>0</v>
@@ -1953,88 +1953,88 @@
         <v>25</v>
       </c>
       <c r="B25" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C25">
         <v>1</v>
       </c>
       <c r="D25" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E25">
         <v>0</v>
       </c>
       <c r="F25" t="s">
+        <v>240</v>
+      </c>
+      <c r="G25" t="s">
+        <v>234</v>
+      </c>
+      <c r="H25" t="s">
         <v>241</v>
       </c>
-      <c r="G25" t="s">
+      <c r="I25" t="s">
         <v>235</v>
       </c>
-      <c r="H25" t="s">
-        <v>242</v>
-      </c>
-      <c r="I25" t="s">
+      <c r="J25" t="s">
+        <v>244</v>
+      </c>
+      <c r="K25" t="s">
+        <v>198</v>
+      </c>
+      <c r="L25" t="s">
+        <v>245</v>
+      </c>
+      <c r="M25" t="s">
         <v>236</v>
       </c>
-      <c r="J25" t="s">
-        <v>245</v>
-      </c>
-      <c r="K25" t="s">
+      <c r="N25" t="s">
+        <v>247</v>
+      </c>
+      <c r="O25" t="s">
+        <v>248</v>
+      </c>
+      <c r="P25" t="s">
+        <v>249</v>
+      </c>
+      <c r="Q25" t="s">
+        <v>246</v>
+      </c>
+      <c r="R25" t="s">
+        <v>251</v>
+      </c>
+      <c r="S25" t="s">
+        <v>252</v>
+      </c>
+      <c r="T25" t="s">
         <v>199</v>
       </c>
-      <c r="L25" t="s">
+      <c r="U25" t="s">
+        <v>250</v>
+      </c>
+      <c r="V25" t="s">
         <v>246</v>
       </c>
-      <c r="M25" t="s">
-        <v>237</v>
-      </c>
-      <c r="N25" t="s">
-        <v>248</v>
-      </c>
-      <c r="O25" t="s">
-        <v>249</v>
-      </c>
-      <c r="P25" t="s">
-        <v>250</v>
-      </c>
-      <c r="Q25" t="s">
-        <v>247</v>
-      </c>
-      <c r="R25" t="s">
-        <v>252</v>
-      </c>
-      <c r="S25" t="s">
+      <c r="W25" t="s">
         <v>253</v>
       </c>
-      <c r="T25" t="s">
-        <v>200</v>
-      </c>
-      <c r="U25" t="s">
-        <v>251</v>
-      </c>
-      <c r="V25" t="s">
-        <v>247</v>
-      </c>
-      <c r="W25" t="s">
-        <v>254</v>
-      </c>
       <c r="X25" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="Y25" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="Z25" t="s">
+        <v>369</v>
+      </c>
+      <c r="AA25" t="s">
+        <v>368</v>
+      </c>
+      <c r="AB25" t="s">
         <v>370</v>
       </c>
-      <c r="AA25" t="s">
-        <v>369</v>
-      </c>
-      <c r="AB25" t="s">
-        <v>371</v>
-      </c>
       <c r="AC25" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
     </row>
     <row r="26" spans="1:30" x14ac:dyDescent="0.25">
@@ -2048,85 +2048,85 @@
         <v>2</v>
       </c>
       <c r="D26" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="E26">
         <v>1</v>
       </c>
       <c r="F26" t="s">
+        <v>254</v>
+      </c>
+      <c r="G26" t="s">
         <v>255</v>
       </c>
-      <c r="G26" t="s">
+      <c r="H26" t="s">
         <v>256</v>
       </c>
-      <c r="H26" t="s">
-        <v>257</v>
-      </c>
       <c r="I26" t="s">
+        <v>259</v>
+      </c>
+      <c r="J26" t="s">
+        <v>271</v>
+      </c>
+      <c r="K26" t="s">
+        <v>266</v>
+      </c>
+      <c r="L26" t="s">
         <v>260</v>
       </c>
-      <c r="J26" t="s">
-        <v>272</v>
-      </c>
-      <c r="K26" t="s">
+      <c r="M26" t="s">
+        <v>265</v>
+      </c>
+      <c r="N26" t="s">
+        <v>261</v>
+      </c>
+      <c r="O26" t="s">
+        <v>263</v>
+      </c>
+      <c r="P26" t="s">
+        <v>262</v>
+      </c>
+      <c r="Q26" t="s">
         <v>267</v>
       </c>
-      <c r="L26" t="s">
-        <v>261</v>
-      </c>
-      <c r="M26" t="s">
-        <v>266</v>
-      </c>
-      <c r="N26" t="s">
-        <v>262</v>
-      </c>
-      <c r="O26" t="s">
+      <c r="R26" t="s">
         <v>264</v>
       </c>
-      <c r="P26" t="s">
+      <c r="S26" t="s">
+        <v>268</v>
+      </c>
+      <c r="T26" t="s">
+        <v>269</v>
+      </c>
+      <c r="U26" t="s">
+        <v>270</v>
+      </c>
+      <c r="V26" t="s">
         <v>263</v>
       </c>
-      <c r="Q26" t="s">
-        <v>268</v>
-      </c>
-      <c r="R26" t="s">
-        <v>265</v>
-      </c>
-      <c r="S26" t="s">
-        <v>269</v>
-      </c>
-      <c r="T26" t="s">
-        <v>270</v>
-      </c>
-      <c r="U26" t="s">
-        <v>271</v>
-      </c>
-      <c r="V26" t="s">
-        <v>264</v>
-      </c>
       <c r="W26" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="X26" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="Y26" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="Z26" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="AA26" t="s">
+        <v>354</v>
+      </c>
+      <c r="AB26" t="s">
         <v>355</v>
       </c>
-      <c r="AB26" t="s">
-        <v>356</v>
-      </c>
       <c r="AC26" t="s">
+        <v>396</v>
+      </c>
+      <c r="AD26" t="s">
         <v>397</v>
-      </c>
-      <c r="AD26" t="s">
-        <v>398</v>
       </c>
     </row>
     <row r="27" spans="1:30" x14ac:dyDescent="0.25">
@@ -2140,58 +2140,58 @@
         <v>3</v>
       </c>
       <c r="D27" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E27">
         <v>2</v>
       </c>
       <c r="F27" t="s">
+        <v>201</v>
+      </c>
+      <c r="G27" t="s">
+        <v>258</v>
+      </c>
+      <c r="H27" t="s">
+        <v>209</v>
+      </c>
+      <c r="I27" t="s">
+        <v>275</v>
+      </c>
+      <c r="J27" t="s">
+        <v>276</v>
+      </c>
+      <c r="K27" t="s">
+        <v>277</v>
+      </c>
+      <c r="L27" t="s">
         <v>202</v>
       </c>
-      <c r="G27" t="s">
-        <v>259</v>
-      </c>
-      <c r="H27" t="s">
-        <v>210</v>
-      </c>
-      <c r="I27" t="s">
-        <v>276</v>
-      </c>
-      <c r="J27" t="s">
-        <v>277</v>
-      </c>
-      <c r="K27" t="s">
+      <c r="M27" t="s">
         <v>278</v>
       </c>
-      <c r="L27" t="s">
-        <v>203</v>
-      </c>
-      <c r="M27" t="s">
+      <c r="N27" t="s">
         <v>279</v>
       </c>
-      <c r="N27" t="s">
+      <c r="O27" t="s">
         <v>280</v>
       </c>
-      <c r="O27" t="s">
+      <c r="P27" t="s">
+        <v>283</v>
+      </c>
+      <c r="Q27" t="s">
         <v>281</v>
       </c>
-      <c r="P27" t="s">
-        <v>284</v>
-      </c>
-      <c r="Q27" t="s">
+      <c r="R27" t="s">
         <v>282</v>
       </c>
-      <c r="R27" t="s">
-        <v>283</v>
-      </c>
       <c r="S27" t="s">
+        <v>287</v>
+      </c>
+      <c r="T27" t="s">
         <v>288</v>
       </c>
-      <c r="T27" t="s">
-        <v>289</v>
-      </c>
       <c r="U27" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
     <row r="28" spans="1:30" x14ac:dyDescent="0.25">
@@ -2205,49 +2205,49 @@
         <v>4</v>
       </c>
       <c r="D28" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="E28">
         <v>3</v>
       </c>
       <c r="F28" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="G28" t="s">
+        <v>292</v>
+      </c>
+      <c r="H28" t="s">
         <v>293</v>
       </c>
-      <c r="H28" t="s">
+      <c r="I28" t="s">
+        <v>295</v>
+      </c>
+      <c r="J28" t="s">
         <v>294</v>
       </c>
-      <c r="I28" t="s">
+      <c r="K28" t="s">
+        <v>301</v>
+      </c>
+      <c r="L28" t="s">
+        <v>302</v>
+      </c>
+      <c r="M28" t="s">
         <v>296</v>
       </c>
-      <c r="J28" t="s">
-        <v>295</v>
-      </c>
-      <c r="K28" t="s">
-        <v>302</v>
-      </c>
-      <c r="L28" t="s">
+      <c r="N28" t="s">
+        <v>297</v>
+      </c>
+      <c r="O28" t="s">
+        <v>211</v>
+      </c>
+      <c r="P28" t="s">
         <v>303</v>
       </c>
-      <c r="M28" t="s">
-        <v>297</v>
-      </c>
-      <c r="N28" t="s">
+      <c r="Q28" t="s">
+        <v>304</v>
+      </c>
+      <c r="R28" t="s">
         <v>298</v>
-      </c>
-      <c r="O28" t="s">
-        <v>212</v>
-      </c>
-      <c r="P28" t="s">
-        <v>304</v>
-      </c>
-      <c r="Q28" t="s">
-        <v>305</v>
-      </c>
-      <c r="R28" t="s">
-        <v>299</v>
       </c>
     </row>
     <row r="29" spans="1:30" x14ac:dyDescent="0.25">
@@ -2261,34 +2261,34 @@
         <v>5</v>
       </c>
       <c r="D29" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="E29">
         <v>4</v>
       </c>
       <c r="F29" t="s">
+        <v>299</v>
+      </c>
+      <c r="G29" t="s">
+        <v>212</v>
+      </c>
+      <c r="H29" t="s">
+        <v>213</v>
+      </c>
+      <c r="I29" t="s">
         <v>300</v>
       </c>
-      <c r="G29" t="s">
-        <v>213</v>
-      </c>
-      <c r="H29" t="s">
+      <c r="J29" t="s">
+        <v>215</v>
+      </c>
+      <c r="K29" t="s">
         <v>214</v>
       </c>
-      <c r="I29" t="s">
-        <v>301</v>
-      </c>
-      <c r="J29" t="s">
-        <v>216</v>
-      </c>
-      <c r="K29" t="s">
-        <v>215</v>
-      </c>
       <c r="L29" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="M29" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="30" spans="1:30" x14ac:dyDescent="0.25">
@@ -2302,43 +2302,43 @@
         <v>6</v>
       </c>
       <c r="D30" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="E30">
         <v>5</v>
       </c>
       <c r="F30" t="s">
+        <v>310</v>
+      </c>
+      <c r="G30" t="s">
+        <v>320</v>
+      </c>
+      <c r="H30" t="s">
+        <v>216</v>
+      </c>
+      <c r="I30" t="s">
         <v>311</v>
       </c>
-      <c r="G30" t="s">
+      <c r="J30" t="s">
+        <v>217</v>
+      </c>
+      <c r="K30" t="s">
+        <v>312</v>
+      </c>
+      <c r="L30" t="s">
+        <v>218</v>
+      </c>
+      <c r="M30" t="s">
+        <v>219</v>
+      </c>
+      <c r="N30" t="s">
+        <v>313</v>
+      </c>
+      <c r="O30" t="s">
         <v>321</v>
       </c>
-      <c r="H30" t="s">
-        <v>217</v>
-      </c>
-      <c r="I30" t="s">
-        <v>312</v>
-      </c>
-      <c r="J30" t="s">
-        <v>218</v>
-      </c>
-      <c r="K30" t="s">
-        <v>313</v>
-      </c>
-      <c r="L30" t="s">
-        <v>219</v>
-      </c>
-      <c r="M30" t="s">
-        <v>220</v>
-      </c>
-      <c r="N30" t="s">
-        <v>314</v>
-      </c>
-      <c r="O30" t="s">
-        <v>322</v>
-      </c>
       <c r="P30" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
     <row r="31" spans="1:30" x14ac:dyDescent="0.25">
@@ -2352,67 +2352,67 @@
         <v>7</v>
       </c>
       <c r="D31" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="E31">
         <v>6</v>
       </c>
       <c r="F31" t="s">
+        <v>314</v>
+      </c>
+      <c r="G31" t="s">
+        <v>220</v>
+      </c>
+      <c r="H31" t="s">
         <v>315</v>
       </c>
-      <c r="G31" t="s">
-        <v>221</v>
-      </c>
-      <c r="H31" t="s">
+      <c r="I31" t="s">
+        <v>222</v>
+      </c>
+      <c r="J31" t="s">
         <v>316</v>
       </c>
-      <c r="I31" t="s">
-        <v>223</v>
-      </c>
-      <c r="J31" t="s">
+      <c r="K31" t="s">
         <v>317</v>
       </c>
-      <c r="K31" t="s">
+      <c r="L31" t="s">
         <v>318</v>
       </c>
-      <c r="L31" t="s">
-        <v>319</v>
-      </c>
       <c r="M31" t="s">
+        <v>356</v>
+      </c>
+      <c r="N31" t="s">
         <v>357</v>
       </c>
-      <c r="N31" t="s">
+      <c r="O31" t="s">
         <v>358</v>
       </c>
-      <c r="O31" t="s">
+      <c r="P31" t="s">
         <v>359</v>
       </c>
-      <c r="P31" t="s">
+      <c r="Q31" t="s">
         <v>360</v>
       </c>
-      <c r="Q31" t="s">
+      <c r="R31" t="s">
         <v>361</v>
       </c>
-      <c r="R31" t="s">
+      <c r="S31" t="s">
         <v>362</v>
       </c>
-      <c r="S31" t="s">
+      <c r="T31" t="s">
         <v>363</v>
       </c>
-      <c r="T31" t="s">
+      <c r="U31" t="s">
         <v>364</v>
       </c>
-      <c r="U31" t="s">
+      <c r="V31" t="s">
         <v>365</v>
       </c>
-      <c r="V31" t="s">
+      <c r="W31" t="s">
         <v>366</v>
       </c>
-      <c r="W31" t="s">
+      <c r="X31" t="s">
         <v>367</v>
-      </c>
-      <c r="X31" t="s">
-        <v>368</v>
       </c>
     </row>
     <row r="32" spans="1:30" x14ac:dyDescent="0.25">
@@ -2426,85 +2426,85 @@
         <v>8</v>
       </c>
       <c r="D32" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="E32">
         <v>7</v>
       </c>
       <c r="F32" t="s">
+        <v>325</v>
+      </c>
+      <c r="G32" t="s">
+        <v>371</v>
+      </c>
+      <c r="H32" t="s">
+        <v>231</v>
+      </c>
+      <c r="I32" t="s">
+        <v>224</v>
+      </c>
+      <c r="J32" t="s">
+        <v>225</v>
+      </c>
+      <c r="K32" t="s">
         <v>326</v>
       </c>
-      <c r="G32" t="s">
-        <v>372</v>
-      </c>
-      <c r="H32" t="s">
-        <v>232</v>
-      </c>
-      <c r="I32" t="s">
-        <v>225</v>
-      </c>
-      <c r="J32" t="s">
-        <v>226</v>
-      </c>
-      <c r="K32" t="s">
+      <c r="L32" t="s">
         <v>327</v>
       </c>
-      <c r="L32" t="s">
+      <c r="M32" t="s">
         <v>328</v>
       </c>
-      <c r="M32" t="s">
+      <c r="N32" t="s">
         <v>329</v>
       </c>
-      <c r="N32" t="s">
+      <c r="O32" t="s">
+        <v>331</v>
+      </c>
+      <c r="P32" t="s">
         <v>330</v>
       </c>
-      <c r="O32" t="s">
+      <c r="Q32" t="s">
+        <v>375</v>
+      </c>
+      <c r="R32" t="s">
+        <v>376</v>
+      </c>
+      <c r="S32" t="s">
         <v>332</v>
       </c>
-      <c r="P32" t="s">
-        <v>331</v>
-      </c>
-      <c r="Q32" t="s">
-        <v>376</v>
-      </c>
-      <c r="R32" t="s">
+      <c r="T32" t="s">
+        <v>333</v>
+      </c>
+      <c r="U32" t="s">
+        <v>334</v>
+      </c>
+      <c r="V32" t="s">
+        <v>335</v>
+      </c>
+      <c r="W32" t="s">
         <v>377</v>
       </c>
-      <c r="S32" t="s">
-        <v>333</v>
-      </c>
-      <c r="T32" t="s">
-        <v>334</v>
-      </c>
-      <c r="U32" t="s">
-        <v>335</v>
-      </c>
-      <c r="V32" t="s">
+      <c r="X32" t="s">
         <v>336</v>
       </c>
-      <c r="W32" t="s">
+      <c r="Y32" t="s">
+        <v>337</v>
+      </c>
+      <c r="Z32" t="s">
+        <v>338</v>
+      </c>
+      <c r="AA32" t="s">
+        <v>339</v>
+      </c>
+      <c r="AB32" t="s">
         <v>378</v>
       </c>
-      <c r="X32" t="s">
-        <v>337</v>
-      </c>
-      <c r="Y32" t="s">
-        <v>338</v>
-      </c>
-      <c r="Z32" t="s">
-        <v>339</v>
-      </c>
-      <c r="AA32" t="s">
+      <c r="AC32" t="s">
         <v>340</v>
       </c>
-      <c r="AB32" t="s">
-        <v>379</v>
-      </c>
-      <c r="AC32" t="s">
+      <c r="AD32" t="s">
         <v>341</v>
-      </c>
-      <c r="AD32" t="s">
-        <v>342</v>
       </c>
     </row>
     <row r="33" spans="1:20" x14ac:dyDescent="0.25">
@@ -2518,55 +2518,55 @@
         <v>9</v>
       </c>
       <c r="D33" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="E33" s="1">
         <v>8</v>
       </c>
       <c r="F33" t="s">
+        <v>342</v>
+      </c>
+      <c r="G33" t="s">
         <v>343</v>
       </c>
-      <c r="G33" t="s">
+      <c r="H33" t="s">
         <v>344</v>
       </c>
-      <c r="H33" t="s">
+      <c r="I33" t="s">
         <v>345</v>
       </c>
-      <c r="I33" t="s">
+      <c r="J33" t="s">
         <v>346</v>
       </c>
-      <c r="J33" t="s">
+      <c r="K33" t="s">
         <v>347</v>
       </c>
-      <c r="K33" t="s">
+      <c r="L33" t="s">
         <v>348</v>
       </c>
-      <c r="L33" t="s">
+      <c r="M33" t="s">
         <v>349</v>
       </c>
-      <c r="M33" t="s">
+      <c r="N33" t="s">
         <v>350</v>
       </c>
-      <c r="N33" t="s">
+      <c r="O33" t="s">
+        <v>325</v>
+      </c>
+      <c r="P33" t="s">
         <v>351</v>
       </c>
-      <c r="O33" t="s">
-        <v>326</v>
-      </c>
-      <c r="P33" t="s">
-        <v>352</v>
-      </c>
       <c r="Q33" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="R33" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="S33" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="T33" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="34" spans="1:20" x14ac:dyDescent="0.25">
@@ -2580,22 +2580,22 @@
         <v>10</v>
       </c>
       <c r="D34" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="K34" t="s">
+        <v>401</v>
+      </c>
+      <c r="L34" t="s">
         <v>402</v>
       </c>
-      <c r="L34" t="s">
+      <c r="M34" t="s">
         <v>403</v>
       </c>
-      <c r="M34" t="s">
+      <c r="N34" t="s">
         <v>404</v>
-      </c>
-      <c r="N34" t="s">
-        <v>405</v>
       </c>
     </row>
     <row r="35" spans="1:20" x14ac:dyDescent="0.25">
@@ -2609,7 +2609,7 @@
         <v>11</v>
       </c>
       <c r="D35" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="36" spans="1:20" x14ac:dyDescent="0.25">
@@ -2623,7 +2623,7 @@
         <v>12</v>
       </c>
       <c r="D36" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="37" spans="1:20" x14ac:dyDescent="0.25">
@@ -2631,13 +2631,13 @@
         <v>37</v>
       </c>
       <c r="B37" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="C37">
         <v>13</v>
       </c>
       <c r="D37" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="38" spans="1:20" x14ac:dyDescent="0.25">
@@ -2645,13 +2645,13 @@
         <v>39</v>
       </c>
       <c r="B38" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C38">
         <v>14</v>
       </c>
       <c r="D38" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="39" spans="1:20" x14ac:dyDescent="0.25">
@@ -2665,7 +2665,7 @@
         <v>15</v>
       </c>
       <c r="D39" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="40" spans="1:20" x14ac:dyDescent="0.25">
@@ -2679,7 +2679,7 @@
         <v>16</v>
       </c>
       <c r="D40" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="41" spans="1:20" x14ac:dyDescent="0.25">
@@ -2693,7 +2693,7 @@
         <v>17</v>
       </c>
       <c r="D41" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="42" spans="1:20" x14ac:dyDescent="0.25">
@@ -2707,7 +2707,7 @@
         <v>18</v>
       </c>
       <c r="D42" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="43" spans="1:20" x14ac:dyDescent="0.25">
@@ -2721,7 +2721,7 @@
         <v>19</v>
       </c>
       <c r="D43" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="44" spans="1:20" x14ac:dyDescent="0.25">
@@ -2735,7 +2735,7 @@
         <v>20</v>
       </c>
       <c r="D44" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="45" spans="1:20" x14ac:dyDescent="0.25">
@@ -2749,7 +2749,7 @@
         <v>21</v>
       </c>
       <c r="D45" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="46" spans="1:20" x14ac:dyDescent="0.25">
@@ -2763,7 +2763,7 @@
         <v>22</v>
       </c>
       <c r="D46" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="47" spans="1:20" x14ac:dyDescent="0.25">
@@ -2777,7 +2777,7 @@
         <v>23</v>
       </c>
       <c r="D47" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="48" spans="1:20" x14ac:dyDescent="0.25">
@@ -2791,7 +2791,7 @@
         <v>24</v>
       </c>
       <c r="D48" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
@@ -2805,7 +2805,7 @@
         <v>25</v>
       </c>
       <c r="D49" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
@@ -2819,7 +2819,7 @@
         <v>26</v>
       </c>
       <c r="D50" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
@@ -2827,13 +2827,13 @@
         <v>49</v>
       </c>
       <c r="B51" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="C51">
         <v>27</v>
       </c>
       <c r="D51" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
@@ -2841,13 +2841,13 @@
         <v>50</v>
       </c>
       <c r="B52" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="C52">
         <v>28</v>
       </c>
       <c r="D52" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
@@ -2861,7 +2861,7 @@
         <v>29</v>
       </c>
       <c r="D53" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
@@ -2875,7 +2875,7 @@
         <v>30</v>
       </c>
       <c r="D54" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
@@ -2889,7 +2889,7 @@
         <v>31</v>
       </c>
       <c r="D55" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
@@ -2903,7 +2903,7 @@
         <v>32</v>
       </c>
       <c r="D56" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
@@ -2917,7 +2917,7 @@
         <v>33</v>
       </c>
       <c r="D57" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
@@ -2925,13 +2925,13 @@
         <v>58</v>
       </c>
       <c r="B58" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="C58">
         <v>34</v>
       </c>
       <c r="D58" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
@@ -2939,13 +2939,13 @@
         <v>61</v>
       </c>
       <c r="B59" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C59">
         <v>35</v>
       </c>
       <c r="D59" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
@@ -2959,7 +2959,7 @@
         <v>36</v>
       </c>
       <c r="D60" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
@@ -2991,7 +2991,7 @@
         <v>64</v>
       </c>
       <c r="B64" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.25">
@@ -3213,7 +3213,7 @@
     </row>
     <row r="97" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B97" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="98" spans="2:2" x14ac:dyDescent="0.25">
@@ -3303,7 +3303,7 @@
     </row>
     <row r="115" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B115" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="116" spans="2:2" x14ac:dyDescent="0.25">
@@ -3328,7 +3328,7 @@
     </row>
     <row r="120" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B120" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="121" spans="2:2" x14ac:dyDescent="0.25">
@@ -3343,7 +3343,7 @@
     </row>
     <row r="123" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B123" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="124" spans="2:2" x14ac:dyDescent="0.25">
@@ -3358,7 +3358,7 @@
     </row>
     <row r="126" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B126" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="127" spans="2:2" x14ac:dyDescent="0.25">
@@ -3403,7 +3403,7 @@
     </row>
     <row r="135" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B135" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="136" spans="2:2" x14ac:dyDescent="0.25">
@@ -3418,92 +3418,92 @@
     </row>
     <row r="138" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B138" t="s">
-        <v>192</v>
+        <v>407</v>
       </c>
     </row>
     <row r="139" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B139" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="140" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B140" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="141" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B141" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="142" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B142" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="143" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B143" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="144" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B144" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="145" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B145" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="146" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B146" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="147" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B147" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="148" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B148" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="149" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B149" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="150" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B150" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="151" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B151" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="152" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B152" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="153" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B153" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="154" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B154" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="155" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B155" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
New sprites, pre champion cutscene and Hall of Fame done!
</commit_message>
<xml_diff>
--- a/stuff/xhenos story work.xlsx
+++ b/stuff/xhenos story work.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\git\PokemonXhenos\stuff\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC8EA829-FD4E-4FBA-B8ED-E851A110DBD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1492003D-2BBC-420B-9EB0-F96D0B8E165C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{271A13BE-4517-4656-AED4-3C6BEDDB1427}"/>
   </bookViews>
@@ -16,6 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="446" uniqueCount="408">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="447" uniqueCount="409">
   <si>
     <t>Current</t>
   </si>
@@ -1260,6 +1261,9 @@
   </si>
   <si>
     <t>Then Nova pulls up to personally thank you guys for setting her free and you all go into the champion room</t>
+  </si>
+  <si>
+    <t>Champ Scene</t>
   </si>
 </sst>
 </file>
@@ -2507,7 +2511,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="33" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>33</v>
       </c>
@@ -2568,8 +2572,11 @@
       <c r="T33" t="s">
         <v>406</v>
       </c>
-    </row>
-    <row r="34" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="U33" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="34" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>34</v>
       </c>
@@ -2598,7 +2605,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="35" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>35</v>
       </c>
@@ -2612,7 +2619,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="36" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>36</v>
       </c>
@@ -2626,7 +2633,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="37" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>37</v>
       </c>
@@ -2640,7 +2647,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="38" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>39</v>
       </c>
@@ -2654,7 +2661,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="39" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>38</v>
       </c>
@@ -2668,7 +2675,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="40" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>40</v>
       </c>
@@ -2682,7 +2689,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="41" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>41</v>
       </c>
@@ -2696,7 +2703,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="42" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>42</v>
       </c>
@@ -2710,7 +2717,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="43" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>45</v>
       </c>
@@ -2724,7 +2731,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="44" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>43</v>
       </c>
@@ -2738,7 +2745,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="45" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>44</v>
       </c>
@@ -2752,7 +2759,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="46" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>46</v>
       </c>
@@ -2766,7 +2773,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="47" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>47</v>
       </c>
@@ -2780,7 +2787,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="48" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>51</v>
       </c>

</xml_diff>

<commit_message>
Added some postgame stuff:
Catching the other legendary and Merlin's staff!
</commit_message>
<xml_diff>
--- a/stuff/xhenos story work.xlsx
+++ b/stuff/xhenos story work.xlsx
@@ -2,21 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\git\PokemonXhenos\stuff\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1492003D-2BBC-420B-9EB0-F96D0B8E165C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E30B02BE-F8AE-49F3-BBDA-9C02B8BCF122}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{271A13BE-4517-4656-AED4-3C6BEDDB1427}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{271A13BE-4517-4656-AED4-3C6BEDDB1427}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="447" uniqueCount="409">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="443" uniqueCount="405">
   <si>
     <t>Current</t>
   </si>
@@ -1179,9 +1178,6 @@
     <t>In order to summon Dragowrath to catch, the player must get Merlin's staff (from the final room of the gauntlet they chose and captured one of the dragon's at)</t>
   </si>
   <si>
-    <t>The staff appears after the player gets back from outer space and saves Earth</t>
-  </si>
-  <si>
     <t>Once they beat Arthra in the Elite Four, she has dialogue that says that she'll set her dragon free (for the player to catch), it goes back to its original resting place (other gauntlet)</t>
   </si>
   <si>
@@ -1242,18 +1238,6 @@
     <t>Rick Pad</t>
   </si>
   <si>
-    <t>Whiskeroar</t>
-  </si>
-  <si>
-    <t>Chlorie</t>
-  </si>
-  <si>
-    <t>Astrid</t>
-  </si>
-  <si>
-    <t>Arthra</t>
-  </si>
-  <si>
     <t>Necrozma can be obtained once the player rematches the league and wins again, then after beating Ryder again he will have Necrozma call more of its kind by the ship in space</t>
   </si>
   <si>
@@ -1264,6 +1248,9 @@
   </si>
   <si>
     <t>Champ Scene</t>
+  </si>
+  <si>
+    <t>The staff appears after the player becomes champion</t>
   </si>
 </sst>
 </file>
@@ -2038,7 +2025,7 @@
         <v>370</v>
       </c>
       <c r="AC25" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="26" spans="1:30" x14ac:dyDescent="0.25">
@@ -2127,10 +2114,10 @@
         <v>355</v>
       </c>
       <c r="AC26" t="s">
+        <v>395</v>
+      </c>
+      <c r="AD26" t="s">
         <v>396</v>
-      </c>
-      <c r="AD26" t="s">
-        <v>397</v>
       </c>
     </row>
     <row r="27" spans="1:30" x14ac:dyDescent="0.25">
@@ -2195,7 +2182,7 @@
         <v>288</v>
       </c>
       <c r="U27" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="28" spans="1:30" x14ac:dyDescent="0.25">
@@ -2289,10 +2276,10 @@
         <v>214</v>
       </c>
       <c r="L29" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="M29" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="30" spans="1:30" x14ac:dyDescent="0.25">
@@ -2342,7 +2329,7 @@
         <v>321</v>
       </c>
       <c r="P30" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
     </row>
     <row r="31" spans="1:30" x14ac:dyDescent="0.25">
@@ -2561,19 +2548,19 @@
         <v>351</v>
       </c>
       <c r="Q33" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
       <c r="R33" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="S33" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="T33" t="s">
-        <v>406</v>
+        <v>401</v>
       </c>
       <c r="U33" t="s">
-        <v>408</v>
+        <v>403</v>
       </c>
     </row>
     <row r="34" spans="1:21" x14ac:dyDescent="0.25">
@@ -2592,18 +2579,6 @@
       <c r="E34" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="K34" t="s">
-        <v>401</v>
-      </c>
-      <c r="L34" t="s">
-        <v>402</v>
-      </c>
-      <c r="M34" t="s">
-        <v>403</v>
-      </c>
-      <c r="N34" t="s">
-        <v>404</v>
-      </c>
     </row>
     <row r="35" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
@@ -3425,7 +3400,7 @@
     </row>
     <row r="138" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B138" t="s">
-        <v>407</v>
+        <v>402</v>
       </c>
     </row>
     <row r="139" spans="2:2" x14ac:dyDescent="0.25">
@@ -3455,62 +3430,62 @@
     </row>
     <row r="144" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B144" t="s">
-        <v>380</v>
+        <v>404</v>
       </c>
     </row>
     <row r="145" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B145" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="146" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B146" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="147" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B147" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="148" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B148" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="149" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B149" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="150" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B150" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="151" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B151" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="152" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B152" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="153" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B153" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="154" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B154" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="155" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B155" t="s">
-        <v>405</v>
+        <v>400</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Work on UP quest and map transitions
</commit_message>
<xml_diff>
--- a/stuff/xhenos story work.xlsx
+++ b/stuff/xhenos story work.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\git\PokemonXhenos\stuff\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E30B02BE-F8AE-49F3-BBDA-9C02B8BCF122}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1A0FC56-F546-4885-BF29-1E5D2F1737A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{271A13BE-4517-4656-AED4-3C6BEDDB1427}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="443" uniqueCount="405">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="449" uniqueCount="411">
   <si>
     <t>Current</t>
   </si>
@@ -1251,6 +1251,24 @@
   </si>
   <si>
     <t>The staff appears after the player becomes champion</t>
+  </si>
+  <si>
+    <t>Lauryn 1</t>
+  </si>
+  <si>
+    <t>Shae 1</t>
+  </si>
+  <si>
+    <t>Lauryn 2</t>
+  </si>
+  <si>
+    <t>Lauryn 3</t>
+  </si>
+  <si>
+    <t>Lauryn Research</t>
+  </si>
+  <si>
+    <t>Did UP Test</t>
   </si>
 </sst>
 </file>
@@ -2184,6 +2202,24 @@
       <c r="U27" t="s">
         <v>393</v>
       </c>
+      <c r="V27" t="s">
+        <v>405</v>
+      </c>
+      <c r="W27" t="s">
+        <v>406</v>
+      </c>
+      <c r="X27" t="s">
+        <v>407</v>
+      </c>
+      <c r="Y27" t="s">
+        <v>409</v>
+      </c>
+      <c r="Z27" t="s">
+        <v>408</v>
+      </c>
+      <c r="AA27" t="s">
+        <v>410</v>
+      </c>
     </row>
     <row r="28" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A28" t="s">

</xml_diff>

<commit_message>
Tons of work on Excel versions of the docs!
</commit_message>
<xml_diff>
--- a/stuff/xhenos story work.xlsx
+++ b/stuff/xhenos story work.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\git\PokemonXhenos\stuff\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1A0FC56-F546-4885-BF29-1E5D2F1737A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{974AA1AD-F39E-414D-A749-8FF649A5E01A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{271A13BE-4517-4656-AED4-3C6BEDDB1427}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="449" uniqueCount="411">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="896" uniqueCount="410">
   <si>
     <t>Current</t>
   </si>
@@ -1262,13 +1262,10 @@
     <t>Lauryn 2</t>
   </si>
   <si>
-    <t>Lauryn 3</t>
-  </si>
-  <si>
-    <t>Lauryn Research</t>
-  </si>
-  <si>
     <t>Did UP Test</t>
+  </si>
+  <si>
+    <t>Caught UP</t>
   </si>
 </sst>
 </file>
@@ -2212,13 +2209,10 @@
         <v>407</v>
       </c>
       <c r="Y27" t="s">
+        <v>408</v>
+      </c>
+      <c r="Z27" t="s">
         <v>409</v>
-      </c>
-      <c r="Z27" t="s">
-        <v>408</v>
-      </c>
-      <c r="AA27" t="s">
-        <v>410</v>
       </c>
     </row>
     <row r="28" spans="1:30" x14ac:dyDescent="0.25">

</xml_diff>